<commit_message>
Performance: tapping "Since <date>" no longer crashes the screen
Found rendering Build 53 for the Performance step (2026-09-14), and still in the app: the window's words
came from a table with no Since entry, so the summary title read undefined.toUpperCase() and the
screen crashed on the chip the approved design opens on. Its start date also fell through to a year ago.

- phraseFor gives every window its words; Since reads "since Aug 29"
- the Since walk starts at the first recorded day, and its beginning is labelled with that date
- the spoken summary uses the same words
- performance_window_chips.test.tsx taps every chip

Logged as B-96. Still open for the Performance step (workplan): the Since chip's own return is worked
out from today, because startDateFor has no Since case.

Gates: build-all green — 287 suites, 2,821 tests, tsc clean, UI-test gate passing.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -3479,6 +3479,62 @@
       </c>
       <c r="F107" s="2" t="inlineStr"/>
     </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Performance crashed when the "Since &lt;date&gt;" window chip was tapped — in Build 53 and since: the window's words came from a table with no Since entry (undefined.toUpperCase), and its start date fell through to a year ago. Found rendering Build 53 for the Performance step.</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Claude: fixed 2026-09-14 — every window has words (Since reads "since Aug 29"), the Since walk starts where the record starts, the spoken summary uses the same words; performance_window_chips.test.tsx taps every chip.</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>src/screens/PerformanceScreen.tsx (phraseFor, periodStartKey) · src/screens/__tests__/performance_window_chips.test.tsx</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Performance step findings still to take to the founder: (1) the Since chip's OWN return is worked out from today, because startDateFor (MK-PF-F-…, src/domain/performance) has no Since case; (2) with a year's window and 16 days of record, each per-account walk reads $0 for accounts worth $301,610 and $52,704; (3) Build 53 still carries the older Invest sections below the approved design (Your return, Honest comparison, Look ahead / Look back, Your investments list, add/import/record buttons); (4) the account page has no per-account walk, no return per holding and no Total row that the approved design draws.</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Claude: draw Performance as Build 53 shipped it for the founder to confirm, with each of these marked, before any change.</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>TO DO</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/networth-and-performance/archive/2026-08-10_moneykeel_pres_mock_performance_v01.html (approved final) · August 14th Design/design_handoff_net_worth/Performance.dc.html</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
The tracker row for the seven-step re-run — 15 of 17, with the two that remain stated plainly
My previous commit updated the decision log and the code but the tracker row failed on a syntax
error of mine (a trailing comma left a paren unclosed), so the workbook rebuilt from the old JSON and
still said 11 of 17. The row now carries the true state: what closed, what is open, the 139 decisions
cited nowhere in the module's code, and the four errors of my own the run surfaced.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -5894,17 +5894,17 @@
     <row r="183" ht="60" customHeight="1">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>Net worth — his seven steps run end to end, and the Word report</t>
+          <t>Net worth — his seven steps: 15 of 17 pass</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>RUN 2026-10-01 by module-launch-steps.py. 11 of 17 checks PASS, 6 fail. PASS: 2.b (all 48 metrics on the standards), 3.a, 3.b, 3.d (86 tests, 86 pass), 4.a-4.d (8 orchestrators, 56 tests, 56 pass), 5 (0 orphan metrics or functions), 6.a + 6.b (10 use cases, all pass). FAIL: 1.a (Itemize is the only screen without his approval — one word from him); 1.b (118 of 225 decisions unconfirmed, 20 hand readings not pinned by a test); 1.c (138 figures with no identifier across all 7 screens); 2.a (3 metrics never issued, Alternatives figures declared under the MENU family, Add account has no metric, 6 labels hold a description not the screen’s words); 2.c (11 corrections owed, closes with 2.a); 3.c (only 1 of 101 functions is named by its identifier in a test — traceability, not correctness; the 86 door tests do exercise them).</t>
+          <t>RE-RUN 2026-10-01 after working the failures on his "go". 15 of 17 PASS, 2 open. CLOSED THIS PASS: 1.a (the Itemize door decided and built on the Account portfolio, DEC-0651 — it had no door in ANY approved design and was unreachable for bonds and alternatives accounts); 2.a and 2.c (3 metrics issued; the Alternatives figures re-filed from the MENU family to MK-NW-M-049/050 with the menu ids RETIRED not re-pointed; MK-NW-M-051/052 issued and declared for figures the screen shows and nothing described; 3 labels rewritten to the screen’s own words); 3.c (all 101 functions trace to their test in one hop via a generated index); 5 (re-passed after I broke it by issuing two metrics without declaring them — fixing that exposed a real one-door breach: the Alternatives screen was filtering and summing accounts itself while asking the door only for the rate. Every figure on that screen now comes off MK-NW-O-005).</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>REPORTED — 5 of the 6 failures are mine; 1.a needs one word from him.</t>
+          <t>IN PROGRESS — 15 of 17. 1.b and 1.c remain, both mine.</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>STEP 7: NOT launch ready. Order to close: 1.a (him), then 2.a + 2.c, then 1.c, then 3.c, then 1.b which is the long pole. THREE ERRORS OF MINE caught while running it: 2.a’s label matcher rejected labels present on mocks I had drawn an hour earlier (it needed per-word matching, not a contiguous phrase); two of the ten use-case test paths were typed from memory and did not exist; and 1.a first guessed approval from mock FILENAMES instead of reading the one design record.</t>
+          <t>STILL OPEN: 1.b — 90 of 217 decisions unconfirmed, mostly BATCH approvals ("Approve all 25") that must be unpacked before any one ruling can be confirmed against a screen; an index would make them traceable without making them compliant, so the number is left true. 1.c — 138 figures print with no identifier across all 7 screens (NetWorth 51, AccountDetail 31, HoldingDetail 18, Bonds 17, Itemize 11, OtherInvestments 9, AddAccount 1). THE ONE NUMBER WORTH HIS EYE: 139 of the 217 decisions governing this module are cited nowhere in its code — 78 now are, up from about none this morning — so every figure works but a wrong number cannot be traced back to his ruling in one hop. FOUR ERRORS OF MINE, each found by USING the runner rather than reading it: the label classifier called lowercase screen copy a "description"; the string extractor missed JSX text between braces; the function mapper read a comment instead of the declaring file and wrongly reported saveAssets as untested; and 3.c scanned only the nine door tests, so it could not see the index that answers it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Performance: launch ready — all 17 checks pass (his word on Look back v01, DEC-1069)
Recorded in the decision log with its path, the design record, a test and the tracker;
step 1.a now knows the Look back row; the two decision ratchets carry their true numbers
(342 without a path, 23 apparent repeats). Report v02 printed from the run; v01 archived.
Master build and every gate pass; suite 3,157 green.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -5986,17 +5986,17 @@
     <row r="186" ht="60" customHeight="1">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Performance — his seven steps: 16 of 17 pass</t>
+          <t>Performance — his seven steps: 17 of 17 pass</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>ONE THING FOR HIM: the Look back screen has a drawing of record for the first time — moneykeel_pres_mock_look-back_v01.html, drawn 2026-10-01 from the screen's own code with the MoneyKeel bar. One word from him makes step 1.a complete and the module launch ready. Nothing else is open.</t>
+          <t>Nothing for him. To confirm on a TestFlight build: the Performance tab, the Look back screen with its app bar.</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>IN PROGRESS — 16 of 17. Only 1.a remains, and it waits on his word for the Look back drawing (v01).</t>
+          <t>DONE 2026-10-02 — all 17 checks pass; step 7 says launch ready. His word on Look back v01 (DEC-1069) closed 1.a.</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Cash flow · Debts tab brought to its approved drawing (cash-flow_v01, frame 6)
YOUR DEBT leads with the total and what it asks of the month; each debt reads as
drawn ('pay first', '22.90% — the costliest', '3 years left', the amount at the
right); one 'Log a payment' under the list asks which debt; PROGRESS shows what has
been paid down since the first month-end on record this year, and is not drawn
where there is nothing to measure from.
src/screens/__tests__/cashflow_matches_v01.test.tsx holds the frame word for word.

New in the calculation: the paid-down amount and its share (MK-CF-M-074, 075), read
from two recorded totals, each with a worked example.

Kept and named as differences: the payoff plan with the mortgage comparison he
moved here (DEC-0157), each debt's payment and interest, and the way to add a debt.

All four Cash flow tabs now match the drawing. Cash flow passes 17 of 17 steps.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -6092,7 +6092,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>IN PROGRESS — matched and locked by test: Account portfolio, Performance tab (4 phones), Net worth (8 states), Cash flow · This month (frames A, B). NOT YET: Cash flow · Expenses, Income and Debts tabs (frames C to F — the built tabs are an older design), Income screens (v07).</t>
+          <t>IN PROGRESS — matched and locked by test: Account portfolio, Performance tab (4 phones), Net worth (8 states), Cash flow all four tabs (6 frames). NOT YET: the Income screens (income-end-to-end_v07, 17 phones: picker, base pay, bonus and stock, rent, interest and dividends, income manager, filing status, summary) and the two kept editors (Bill calendar v02, Monthly income v02).</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 2026-10-03: Performance tab matched to v17 phones 1, 3, 4, 5 by src/screens/__tests__/perf_matches_v17.test.tsx. 2026-10-03: Net worth matched to v08 in all eight states (networth_matches_v08.test.tsx). Cash flow This month REBUILT to cash-flow_v01 frames A and B (cashflow_matches_v01.test.tsx): it had been showing a hero, a pace line, a budget card, twelve bars and a will-it-last strip that the approved drawing does not have, and no Actual card at all. FOUND, NOT YET BUILT: the Expenses, Income and Debts tabs are still the 2026-07-19 design — the calculations behind the approved one exist in the doors, the screens do not draw them.</t>
+          <t xml:space="preserve"> 2026-10-03: Performance tab matched to v17 phones 1, 3, 4, 5 by src/screens/__tests__/perf_matches_v17.test.tsx. 2026-10-03: Net worth matched to v08 in all eight states (networth_matches_v08.test.tsx). Cash flow This month REBUILT to cash-flow_v01 frames A and B (cashflow_matches_v01.test.tsx): it had been showing a hero, a pace line, a budget card, twelve bars and a will-it-last strip that the approved drawing does not have, and no Actual card at all. FOUND, NOT YET BUILT: the Expenses, Income and Debts tabs are still the 2026-07-19 design — the calculations behind the approved one exist in the doors, the screens do not draw them. 2026-10-03 later: Cash flow Expenses, Income and Debts tabs rebuilt to cash-flow_v01 frames C to F; every named difference is listed in cashflow_matches_v01.test.tsx.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: three open rows from the line-by-line comparison of the Income screens
- the Income summary's take-home total is not the sum of its own rows (rent is
  counted before tax in the row and after tax in the total) — blocks the build
- the Income manager is not the screen the approved drawing shows; summary and base
  pay differ in wording — blocks the build
- the kept editors and the Net worth secondary screens still need their tests

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F189"/>
+  <dimension ref="A1:F192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -6111,8 +6111,92 @@
         </is>
       </c>
     </row>
+    <row r="190" ht="60" customHeight="1">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>Income summary — the take-home total is not the sum of its own rows (rent)</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>FOUND 2026-10-03 comparing the screen with income-end-to-end_v07 frame 16. The rows read Your pay $5,000 · Sam’s pay $3,300 · Rent $1,200 and the total under them reads $9,248, not $9,500. The Rent row is the rent after running costs; the total takes the month from the cash-flow grid, which also takes tax off the rent ($1,200 → $948). The approved drawing says $1,200 lands and the total is $9,500 ("$9,500 a month landing"). Decide in the calculation which is the take-home for rent, make the row and the total the same figure, and carry it to Cash flow’s inflow and Home so no screen disagrees. Function: MK-CF-O-004 incomeSummary (usualMonth) against the monthly income grid.</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — mine. BLOCKS THE BUILD: one card disagreeing with itself is the class of error the accuracy rule exists for.</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/functions/cashflow/income-summary.ts · MoneyKeel/documents/cashflow/moneykeel_pres_mock_income-end-to-end_v07.html frame 16</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr"/>
+    </row>
+    <row r="191" ht="60" customHeight="1">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>Income screens — compare line by line with income-end-to-end_v07 and close the gaps</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>Measured 2026-10-03, not yet built. (1) Income manager (frames 1, 9, 10, 11, 12) is NOT the drawn screen: it shows a gross total and a list; the drawing shows "You entered about 3 sources", one line per source with Edit, and "Anything else?" with the seven sources not picked. (2) Income summary (frames 16, 17): wording differs in five places ("= Inflow (income (take-home) + rent)", "December · with the bonus", the bracket and tax lines, the closing sentence), and the empty state shows $0 with three doors where the drawing shows an em-dash and one. (3) Base pay (frames 2 to 8): close; "‹ Income", two sentences and the onboarding frame to check. (4) Filing status (frames 13 to 15) not yet compared.</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — mine. Blocks the build (the release gate needs the match in every data state).</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/cashflow/moneykeel_pres_mock_income-end-to-end_v07.html · src/testing/mockMatch.ts</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr"/>
+    </row>
+    <row r="192" ht="60" customHeight="1">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Kept editors and the Net worth secondary screens — hold each to its drawing with a word-for-word test</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Bill calendar v02, Monthly income v02, Bonds v02, Other investments v02, Itemize v02, Holding detail v02, Add account by hand v01, Look back v01. Each drawing was made from the build in the last three days, so gaps are unlikely — but none has the test yet, and "unlikely" is not "measured".</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — mine.</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>src/testing/mockMatch.ts · the design record</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F189"/>
+  <autoFilter ref="A1:F192"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Outside pack: brief v04 carries the time-weighted rule; supplement 02 holds the 15 cards changed since supplement 01
- Brief v04 (v03 archived): under Job 1's judging order, the owner rule from his returned note —
  "Every return is a time-weighted return (owner, 2026-10-04). A return made any other way is WRONG."
  The example method under standard finance practice names the time-weighted return, not Modified Dietz.
- to-send/moneykeel_audit_cards_changed-since-sent_02.md: brief v04, then the cards whose function
  changed since supplement 01 — among them MK-NW-O-008 thePerformance, MK-NW-O-003 theNetWorth and
  MK-NW-O-004 theEmergencyFund.
- The 26 files of the pack are untouched: they are as sent.

Gates: file and decision gates exit 0 · 240 logic suites, 2,206 tests pass (no app code changed
since the full run of 351 suites, 3,379 tests).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -6225,7 +6225,7 @@
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>MoneyKeel/documents/audit/outside-test-cases/moneykeel_audit_cards_index_v01.md · moneykeel_audit_brief_outside-test-cases_v03.md · Calculation Module code/scripts/build-outside-test-cards.py · moneykeel_function_rules.json</t>
+          <t>MoneyKeel/documents/audit/outside-test-cases/moneykeel_audit_cards_index_v01.md · moneykeel_audit_brief_outside-test-cases_v04.md · Calculation Module code/scripts/build-outside-test-cards.py · moneykeel_function_rules.json</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
@@ -6235,7 +6235,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>Done first, because a function nobody has described cannot be tested from outside: 150 descriptions written into the code, 14 stale copies of records removed (src/__tests__/guard_function_descriptions.test.ts). THE LIMIT OF THE FIRST PACK IS CLOSED: only 32 of its cards carried any rule. Now 318 of 318 carry the formula in words — how the function gets its answer, every number included — each written by reading the function. Held three ways: a function that changes stops the build until its formula is read again (step B7); 463 figures stated in the formulas are each traced to the function, 7 of them worked by hand and re-checked; no card carries code. Each batch also carries the formulas its cards lean on, and the Cash flow batches carry the published 2026 tax and limit amounts, read from the app, for the models to check against their source. WHAT THIS DOES NOT PROVE: the formulas are my reading of my own code. The outside models judge whether each is the right formula; whether the code does what its formula says is settled only when their cases are run against the app. CORRECTED AFTER SENDING, 2026-10-04: 12 cards in six of the sent files describe a formula that has since been fixed — cashflow 01 (MK-CF-O-001, MK-CF-O-004), cashflow 06 (MK-CF-F-087, MK-CF-F-092), cashflow 11 (MK-CF-F-144, MK-CF-F-146), cashflow 13 (MK-CF-F-180, MK-CF-F-181, MK-CF-F-186), cashflow 15 (MK-CF-F-182), performance 03 (MK-PF-F-010, MK-PF-F-023). A model that calls one of those twelve WRONG is judging the formula as it was sent; its verdict is read against what was then fixed, and the supplement gets the corrected formula judged afresh.</t>
+          <t>Done first, because a function nobody has described cannot be tested from outside: 150 descriptions written into the code, 14 stale copies of records removed (src/__tests__/guard_function_descriptions.test.ts). THE LIMIT OF THE FIRST PACK IS CLOSED: only 32 of its cards carried any rule. Now 318 of 318 carry the formula in words — how the function gets its answer, every number included — each written by reading the function. Held three ways: a function that changes stops the build until its formula is read again (step B7); 463 figures stated in the formulas are each traced to the function, 7 of them worked by hand and re-checked; no card carries code. Each batch also carries the formulas its cards lean on, and the Cash flow batches carry the published 2026 tax and limit amounts, read from the app, for the models to check against their source. WHAT THIS DOES NOT PROVE: the formulas are my reading of my own code. The outside models judge whether each is the right formula; whether the code does what its formula says is settled only when their cases are run against the app. CORRECTED AFTER SENDING, 2026-10-04: 12 cards in six of the sent files describe a formula that has since been fixed — cashflow 01 (MK-CF-O-001, MK-CF-O-004), cashflow 06 (MK-CF-F-087, MK-CF-F-092), cashflow 11 (MK-CF-F-144, MK-CF-F-146), cashflow 13 (MK-CF-F-180, MK-CF-F-181, MK-CF-F-186), cashflow 15 (MK-CF-F-182), performance 03 (MK-PF-F-010, MK-PF-F-023). A model that calls one of those twelve WRONG is judging the formula as it was sent; its verdict is read against what was then fixed, and the supplement gets the corrected formula judged afresh. 2026-10-04, later: brief v04 adds the owner rule "Every return is a time-weighted return (owner, 2026-10-04). A return made any other way is WRONG." (v03 archived). Supplement 02 written: to-send/moneykeel_audit_cards_changed-since-sent_02.md — the 15 cards changed since supplement 01, with brief v04 at its top. The 26 files of the pack are as sent and still carry brief v03 and the old return formula on MK-NW-O-008 and MK-NW-O-003.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: the retirement money and the rate the Plan grows it by, against his words of 2026-10-06
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$217</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F216"/>
+  <dimension ref="A1:F217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -6935,8 +6935,36 @@
       </c>
       <c r="F216" s="2" t="inlineStr"/>
     </row>
+    <row r="217" ht="60" customHeight="1">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>Plan build — the retirement money the Plan grows, and the rate it grows by, checked against his words of 2026-10-06</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>HIS WORDS, 2026-10-06: "Per Plan mockup - NW - primary home - car = retirement." and "all return should be TWR. what is reported 12-month return?" WHAT THE APP DOES TODAY. (1) Retirement money (MK-NW-F-033 retirementEarmarkedValue) = every account except the home lived in, the car driven and a 529, each counted whole unless a share is set — DEBTS ARE NOT TAKEN OFF. Net worth takes debts off, so if his Plan drawing starts from net worth the two differ by the debts. (2) The Plan grows that money by one of three rates chosen in the Plan: the blended benchmark (default — each kind's typical long-run return, weighted by the retirement money in it, MK-NW-F-037), 'your 12-month return' (figures the person TYPES per account as 'reported return (12 mo)', weighted the same way, MK-NW-F-004), or a scenario rate typed. No measured return feeds the Plan. MY RECOMMENDATION for the Plan build: 'your 12-month return' should be the app's own time-weighted one-year return per account (what Performance measures, MK-NW-O-008), typed figures only where the app cannot measure — so his rule that every return is time-weighted reaches the Plan. Not built: the Plan waits for the build after this one.</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — for the Plan build. Nothing changed.</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>src/domain/assets/index.ts (MK-NW-F-033, MK-NW-F-037, MK-NW-F-004) · src/domain/retirement/willItLast.ts (MK-PL-F-067) · src/screens/RetirementCockpit.tsx</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F216"/>
+  <autoFilter ref="A1:F217"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Private equity and hedge funds are not offered in this phase — his ruling of 2026-10-06 (DEC-2334), applied to the two doors that still offered them
Add an account no longer offers "Private stake"; the Alternatives screen's first-day sentence names
crypto, commodities and annuities. A row saved earlier with either kind keeps it when edited. The two
drawings carry the ruling at their top; the test that holds them names the difference (item 17).
3,520 tests green; gates exit 0.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$217</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$218</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F217"/>
+  <dimension ref="A1:F218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -6963,8 +6963,36 @@
       </c>
       <c r="F217" s="2" t="inlineStr"/>
     </row>
+    <row r="218" ht="60" customHeight="1">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>Private equity and hedge funds are not offered in this phase — his ruling of 2026-10-06, applied to the two doors that still offered them</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>HIS WORDS, 2026-10-06: "this phase of app no longer has options for Private Equity and Hedge fund." His ruling of 2026-08-04 (DEC-0045) had trimmed the Net worth add sheet; the Add an account form (built later) still offered "Private stake", and the Alternatives screen's first-day sentence still named both. DONE: the chip is gone; the sentence reads crypto, commodities, annuities; a row saved earlier with either kind keeps it when edited. The two drawings carry the ruling at their top; the test that holds them names the difference (item 17).</t>
+        </is>
+      </c>
+      <c r="C218" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>src/screens/AddAccountScreen.tsx · src/screens/OtherInvestmentsScreen.tsx · src/screens/__tests__/kept_editors_match.test.tsx · the two drawings</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F217"/>
+  <autoFilter ref="A1:F218"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Gemini's final audit of Net worth batch 1: 36 of 36 held; two small fixes (a leap-day purchase, a hand-built account's cash in its inside)
Its thirty cases and nine issues run as tests (outside_networth_01_final_gemini.test.ts): 34 passed
before any change, 36 after. Fixed: MK-PF-F-006 capGains — a share bought on 29 February read
short-term one day too long; MK-NW-O-002 theAccount — the uninvested cash an account built by hand
records is in its inside, the rest under its class. Five of its issues were already so (proved by
test); three were not so (the rate-move figure reprices the bond; the 2026 deduction is the IRS figure;
a mortgage is never matched by balance). Holding detail v02 carries the change at its top.
3,556 tests green; gates exit 0.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$218</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$219</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F218"/>
+  <dimension ref="A1:F219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -6991,8 +6991,36 @@
       </c>
       <c r="F218" s="2" t="inlineStr"/>
     </row>
+    <row r="219" ht="60" customHeight="1">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>Outside review — Gemini's final audit of Net worth batch 1 (returned 2026-10-05): nine issues, thirty cases</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>HIS INSTRUCTION, 2026-10-05: "write another brief for Gemini for NW-01 to conduct one final audit before we move to NW-02." Gemini answered "Ready to Close: No" with nine issues. MEASURED: its thirty cases and nine issues as 36 tests (outside_networth_01_final_gemini.test.ts) — 34 passed before any change, 36 after two small fixes. REAL, FIXED: (6) MK-PF-F-006 capGains — a share bought on 29 February read short-term one day too long (the anniversary rolled to 1 March; it is the last day of February). (2) MK-NW-O-002 theAccount — the uninvested cash an account built by hand records for itself is now in its inside, with the rest under the account's class (the same split Net worth counts by since file 2). ALREADY SO, PROVED BY TEST: (1) a zero-coupon bond gets no rate-move figure and a bond with no maturity date gets no yield to maturity; (3) the time-weighted return measures from the first day something was held and gives no figure for a start below zero — no division by zero; (4) rent at or above essentials draws nothing from cash and shows no months; (5) an alternative worth $0 gives no rate and no growth. NOT SO: (9) the rate-move figure reprices the bond at the new yield — not a straight line, and closer than the duration shortcut it asked for; (7) the 2026 standard deduction $16,100 single / $32,200 married IS the IRS figure (Rev. Proc. 2025-32); (8) a mortgage is matched by its property first, then its name, then only when one property and one mortgage are left — never by balance; two alike are both flagged. Three of its nine named functions by ids that are not theirs (F-010, F-012, F-015); read as the functions it meant. One of its figures differs from the app by design: a linked checking account with a deposit and a withdrawal shows income $0, not no figure — the records are there and none is income.</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>DONE — 36 of 36. Net worth batch 1 is closed on my side; his word closes it.</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/audit/outside-test-cases/returned/NW-01-gemini.md · MoneyKeel/functions/networth-and-performance/outside_networth_01_final_gemini.test.ts</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F218"/>
+  <autoFilter ref="A1:F219"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Post Feedback Sync for batches 1 and 2: two standards written, his two approvals in the decision log, the design Changelog backfilled, the taxonomy spec corrected; the final audit of batch 2 written for Gemini
His question, 2026-10-07: had every file been brought level with what the two batches changed in the
code? No. Done now: the standard "how an account is classed, split, counted and named" and the standard
"how a mortgage, rent and a debt are entered and counted"; fourteen decisions name the standard that
carries them; "Rest I am good with." (DEC-2441) and "NW batch one close." (DEC-2440) recorded; the
Changelog's 54 missing rows since 2026-09-26 written into a dated copy, each anchored to its decision,
and the sweep taught that such a row records a decision rather than minting one; the old taxonomy
spec's cash, bonds and property lines corrected. Gemini's final audit of batch 2: 24 cards.
3,556 tests green; gates exit 0.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$219</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$220</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F219"/>
+  <dimension ref="A1:F220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -6424,7 +6424,7 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>DONE — all 30 of its cases run against the app and pass; its renter case now also works for a real person.</t>
+          <t>CLOSED on his word, 2026-10-07: "NW batch one close."</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>DONE — 73 of its 75 answers are the app's; 2 are held at the app's answer and named on the next row.</t>
+          <t>DONE — 73 of 75 its answers, 2 held and approved by him ("Rest I am good with.", 2026-10-06). Final audit for Gemini written 2026-10-07: to-send/moneykeel_audit_final_networth02_for-gemini_v01.md (24 cards: the 15 of the batch as they stand + 9 changed or added since).</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>DONE — 36 of 36. Net worth batch 1 is closed on my side; his word closes it.</t>
+          <t>CLOSED on his word, 2026-10-07: "NW batch one close." — 36 of 36.</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -7019,8 +7019,36 @@
       </c>
       <c r="F219" s="2" t="inlineStr"/>
     </row>
+    <row r="220" ht="60" customHeight="1">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>Post Feedback Sync, 2026-10-07 — every file brought level with what batches 1 and 2 changed in the code</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>HIS QUESTION, 2026-10-07: "The objective of PFS is to update all files - standards, master calculation, decision-log, screens - to changes we are making directly in code. Have you done that for batch 1 and 2?" HONEST ANSWER: no — the master (printed from the code), the drawings (a change table at the top of six) and the tracker were level; the decision log held his rulings but not his two approvals; no standard carried the classification rules or the housing rulings; the design Changelog had no row since 2026-09-26; and the old taxonomy spec still said the opposite of his 2026-08-04 rule. DONE TODAY: (1) two standards written — how an account is classed, split, counted and named (the batch 2 rules, with DEC-0051, 0092, 0095, 0309, 0343, 0045, 2160, 2163, 2334 named as their source) and how a mortgage, rent and a debt are entered and counted (DEC-1923 to 1926, 1668, 1859); fourteen decisions now name the standard that carries them. (2) The decision log: his two approvals recorded — "Rest I am good with." (2026-10-06, batch 2) and "NW batch one close." (2026-10-07, batch 1). (3) The design Changelog: 52 rows backfilled, one per decision of his since 2026-09-27, in a dated copy (FCC-core-detailed-design-v1.3-2026-10-07.xlsx), each anchored to its decision. (4) docs/finwise-taxonomy-spec.md: its cash, bonds and property lines corrected and pointed at the standard. (5) The master: rebuilt from the code by the gates. STILL TRUE: a code change with no ruling of his reaches the standard and the tracker, and the decision log only when he approves it.</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/standards/moneykeel_calc_spec_how-an-account-is-classed-and-counted_v01.md · moneykeel_calc_spec_mortgage-rent-and-debt_v01.md · docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-10-07.xlsx · docs/finwise-taxonomy-spec.md</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F219"/>
+  <autoFilter ref="A1:F220"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
His approval of every code change, finding and change in Net worth batches 1 and 2 (DEC-2484), recorded in the log, the Changelog, the tracker and the three drawings
"all the code changes, findings and changes - for batch one and two - I approved." Eleven tracker rows
that said "decided by me — one line reverses it" are closed on his word; the change tables at the top
of Net worth v08, Performance v17 and Holding detail v02 say approved. App copy quoted in those tables
is no longer in double quotes, so the sweep does not read it as his words (two artefacts removed).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -6439,7 +6439,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>MEASURED 2026-10-04 at his question ("are these 6 findings not in file?"): the test file run against the app as it stood before the fixes (cd9f0b8) — 13 of 32 failed; against the fixes — 0 fail. All six of its findings were real. Still open: the return (its finding 2 — the app still shows 42.32% where 10.97% is right) and "no figure when the record does not reach back". 2026-10-05, STATE OF THIS FILE: its six findings and its five smaller points are fixed and tested; its four unclear points are decided; the return is time-weighted (10.97%). NOT CLOSED IN REAL USE — its finding on the renter who owns a rented-out house (MK-NW-O-004): the fix tells the home's mortgage from another property's, but no screen yet tells the app that a property is a rental, so the case passes only in its test. It closes with steps 2 and 3 of the row "How a mortgage, rent and a debt are entered and counted" (DEC-1924, DEC-1926, DEC-1923). ALSO LEFT FROM WORK THIS FILE STARTED: share transfers synced before 2026-10-04 carry no direction, so a window holding one still shows no return; a balance typed back-dated is assumed to hold that day's money. ONLY Claude's file has come back for this batch; Gemini's has not been run. 2026-10-05 — the renter who owns a rented-out house: closed. Rent entered for a property on the Income screen is what makes it a rental (DEC-1926), so the app no longer needs a field no screen could set. Its "three places" case was worked from the card as sent; the owner's rule of 2026-10-04 (DEC-1923) changed the formula, so the test keeps its numbers on record and asserts the answer under the rule.</t>
+          <t>MEASURED 2026-10-04 at his question ("are these 6 findings not in file?"): the test file run against the app as it stood before the fixes (cd9f0b8) — 13 of 32 failed; against the fixes — 0 fail. All six of its findings were real. Still open: the return (its finding 2 — the app still shows 42.32% where 10.97% is right) and "no figure when the record does not reach back". 2026-10-05, STATE OF THIS FILE: its six findings and its five smaller points are fixed and tested; its four unclear points are decided; the return is time-weighted (10.97%). NOT CLOSED IN REAL USE — its finding on the renter who owns a rented-out house (MK-NW-O-004): the fix tells the home's mortgage from another property's, but no screen yet tells the app that a property is a rental, so the case passes only in its test. It closes with steps 2 and 3 of the row "How a mortgage, rent and a debt are entered and counted" (DEC-1924, DEC-1926, DEC-1923). ALSO LEFT FROM WORK THIS FILE STARTED: share transfers synced before 2026-10-04 carry no direction, so a window holding one still shows no return; a balance typed back-dated is assumed to hold that day's money. ONLY Claude's file has come back for this batch; Gemini's has not been run. 2026-10-05 — the renter who owns a rented-out house: closed. Rent entered for a property on the Income screen is what makes it a rental (DEC-1926), so the app no longer needs a field no screen could set. Its "three places" case was worked from the card as sent; the owner's rule of 2026-10-04 (DEC-1923) changed the formula, so the test keeps its numbers on record and asserts the answer under the rule. APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
         </is>
       </c>
     </row>
@@ -6535,7 +6535,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>REMOVED 2026-10-04 on his instruction ("work on fixing all 5+4 findings"): modifiedDietzOverWindow (window-return.ts), moneyWeighted.ts whole (5 functions), investableChangePct (history.ts); their tests and probes; seven function numbers retired. The bench page's return card is now time-weighted and was rebuilt. The guard reads the engines too and fails the build if one comes back.</t>
+          <t>REMOVED 2026-10-04 on his instruction ("work on fixing all 5+4 findings"): modifiedDietzOverWindow (window-return.ts), moneyWeighted.ts whole (5 functions), investableChangePct (history.ts); their tests and probes; seven function numbers retired. The bench page's return card is now time-weighted and was rebuilt. The guard reads the engines too and fails the build if one comes back. APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04, on his instruction to fix them. (1) SHARES MOVED IN OR OUT: now counted as money in or out at what they were worth, when the record says which way they went and what they were worth. The sync now stores the direction (it was lost: "in" and "out" both became one type), the rebuilt history respects it, and the walk counts it. STILL REFUSED: share-transfer rows synced BEFORE today carry no direction, so a window containing one still shows no return — the direction cannot be recovered from what was stored. (2) HAND-ENTERED ACCOUNT WITH HOLDINGS: fixed — on rebuilt days between two days it was observed holding exactly the same shares and cash, it is given those shares at each day's close (fillBetweenObservations). Different on the two sides: nothing is filled. (3) THE DOLLAR WALK: fixed — cash or shares transferred in from outside, and an account that joined the record inside the window, count as money put in; the walk and the percent tell one story. (4) A BALANCE TYPED BACK-DATED: unchanged — the record assumes each day's value already holds that day's money. 2026-10-05 — item 1 finished: a share transfer synced before 2026-10-04 is given its direction on the next sync, from the activity the broker reports again; it is never imported twice (ingest.test.ts). Until that sync runs, a window holding such a row still shows no return.</t>
+          <t>2026-10-04, on his instruction to fix them. (1) SHARES MOVED IN OR OUT: now counted as money in or out at what they were worth, when the record says which way they went and what they were worth. The sync now stores the direction (it was lost: "in" and "out" both became one type), the rebuilt history respects it, and the walk counts it. STILL REFUSED: share-transfer rows synced BEFORE today carry no direction, so a window containing one still shows no return — the direction cannot be recovered from what was stored. (2) HAND-ENTERED ACCOUNT WITH HOLDINGS: fixed — on rebuilt days between two days it was observed holding exactly the same shares and cash, it is given those shares at each day's close (fillBetweenObservations). Different on the two sides: nothing is filled. (3) THE DOLLAR WALK: fixed — cash or shares transferred in from outside, and an account that joined the record inside the window, count as money put in; the walk and the percent tell one story. (4) A BALANCE TYPED BACK-DATED: unchanged — the record assumes each day's value already holds that day's money. 2026-10-05 — item 1 finished: a share transfer synced before 2026-10-04 is given its direction on the next sync, from the activity the broker reports again; it is never imported twice (ingest.test.ts). Until that sync runs, a window holding such a row still shows no return. APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>Tests: emergency_fund_rent.test.ts (the four logged-debt cases) · sale_takes_oldest_first.test.ts (4) · kept_editors_match (Bonds line) · outside_networth_01 (bonds named). Drawings Bonds v02 and Holding detail v02 carry a note at the top.</t>
+          <t>Tests: emergency_fund_rent.test.ts (the four logged-debt cases) · sale_takes_oldest_first.test.ts (4) · kept_editors_match (Bonds line) · outside_networth_01 (bonds named). Drawings Bonds v02 and Holding detail v02 carry a note at the top. APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
         </is>
       </c>
     </row>
@@ -6759,7 +6759,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>Not pushed. The two drawings carry the changes at their top, in a second table marked as not his rulings: Net worth v08 (8 lines), Performance v17 (5 lines).</t>
+          <t>Not pushed. The two drawings carry the changes at their top, in a second table marked as not his rulings: Net worth v08 (8 lines), Performance v17 (5 lines). APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
         </is>
       </c>
     </row>
@@ -6789,7 +6789,11 @@
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="F211" s="2" t="inlineStr"/>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
+        </is>
+      </c>
     </row>
     <row r="212" ht="60" customHeight="1">
       <c r="A212" s="2" t="inlineStr">
@@ -6819,7 +6823,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>DECIDED BY ME: Home's figure is the one Performance shows, not Net worth's Investments line — it sits beside Performance's return and opens Performance. To reverse: one line in HomeScreen.tsx.</t>
+          <t>DECIDED BY ME: Home's figure is the one Performance shows, not Net worth's Investments line — it sits beside Performance's return and opens Performance. To reverse: one line in HomeScreen.tsx. APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
         </is>
       </c>
     </row>
@@ -6849,7 +6853,11 @@
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="F213" s="2" t="inlineStr"/>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
+        </is>
+      </c>
     </row>
     <row r="214" ht="60" customHeight="1">
       <c r="A214" s="2" t="inlineStr">
@@ -6877,7 +6885,11 @@
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="F214" s="2" t="inlineStr"/>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
+        </is>
+      </c>
     </row>
     <row r="215" ht="60" customHeight="1">
       <c r="A215" s="2" t="inlineStr">
@@ -6905,7 +6917,11 @@
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="F215" s="2" t="inlineStr"/>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
+        </is>
+      </c>
     </row>
     <row r="216" ht="60" customHeight="1">
       <c r="A216" s="2" t="inlineStr">
@@ -7017,7 +7033,11 @@
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="F219" s="2" t="inlineStr"/>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED BY HIM, 2026-10-07: "all the code changes, findings and changes - for batch one and two - I approved."</t>
+        </is>
+      </c>
     </row>
     <row r="220" ht="60" customHeight="1">
       <c r="A220" s="2" t="inlineStr">

</xml_diff>

<commit_message>
What Post Feedback Sync covers (DEC-2634): every change the outside review brings is his decision — recorded, and held by two new gates
His words, 2026-10-07: "The changes we are making with this audit are also changes I am approving, and
while not my direct feedback - these are findings and changes." Batches 3 and 4 are approved under it;
the drawings' change tables say so; the tracker rows close. The naming standard's PFS section now says
what a sync covers — decision log, Changelog, standard, master, formulas in words, tracker, drawings,
the outside pack — whatever caused the change. Two gates hold it: every function id and file path a
standard names must exist and be live (the guard found four stale lines on its first run, fixed), and
every decision of his since the one-master rule must have its Changelog row or the build stops. His
"no" on a count of accounts with no value is recorded. 3,705 tests green; gates exit 0.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -7080,7 +7080,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>DONE — 72 of its 75 answers are the app's; 3 held (2 on his rule DEC-0100, 1 on the Roth limit). Not yet approved by him.</t>
+          <t>DONE — 72 of its 75 answers are the app's; 3 held and named. APPROVED by him 2026-10-07 (DEC-2634).</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -7112,7 +7112,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>DONE — 71 of its 75 answers are the app's; 4 held and named. Not yet approved by him.</t>
+          <t>DONE — 71 of its 75 answers are the app's; 4 held and named. APPROVED by him 2026-10-07 (DEC-2634); his word on the count of accounts with no value: "no" — not built.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Net worth By class: under each class, each account with its part in that class (his ruling DEC-3146, replacing DEC-2747b)
His words, 2026-10-07: "build it per mockup 07 where under each class you list each account Vanguard-0008
$45000, Chase - 0333 $34000." ledgerGroups (MK-NW-F-094) now lists an account under every class it has a
part in, at that part, so the rows under a heading add up to it; the step-by-step setup list prints that
part under the account's name. The main Net worth list already did this. Decision log, Changelog,
standard §10, drawing v08 note, tracker updated. 4,079 tests green; gates exit 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$224</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$225</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F224"/>
+  <dimension ref="A1:F225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7195,8 +7195,40 @@
         </is>
       </c>
     </row>
+    <row r="225" ht="60" customHeight="1">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>Net worth By class: each account under each class with its part (his ruling, DEC-3146)</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>His words, 2026-10-07: "build it per mockup 07 where under each class you list each account Vanguard-0008 $45000, Chase - 0333 $34000." The main Net worth list already did this; MK-NW-F-094 ledgerGroups and the step-by-step setup list did not (a split account sat once under its largest class at its whole balance). Fixed: rows carry each account's part; the setup list prints the part under the account's name. The batch 4 rule DEC-2747b is marked replaced.</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>DONE — test: the rows under each heading add up to it.</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/functions/networth-and-performance/net-worth.ts MK-NW-F-094 · src/screens/NetWorthScreen.tsx · outside_networth_04_final.test.ts</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>Not pushed. Drawing v08's batch 4 line struck through and marked replaced.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F224"/>
+  <autoFilter ref="A1:F225"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Home's YOUR INVESTMENTS is Net worth's Investments line — cash not included (his definition DEC-0457)
MK-XS-M-003 is one figure on Home and Net worth: stocks, funds, bonds and alternatives. Since 2026-10-05
Home printed Performance's ending value instead — the investment accounts whole, their uninvested cash
included — so Home read $355,152 where Net worth read $354,314 (Vanguard's $838 of cash). That was my
batch 2 choice against his definition; its decision row (DEC-2484p) is marked replaced by DEC-0457.
Performance's Ending value is unchanged and keeps its own name. 4,081 tests green; gates exit 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$225</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$226</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F225"/>
+  <dimension ref="A1:F226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7227,8 +7227,40 @@
         </is>
       </c>
     </row>
+    <row r="226" ht="60" customHeight="1">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>Home's YOUR INVESTMENTS = Net worth's Investments line (DEC-0457, MK-XS-M-003)</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>Re-check 2026-10-08. Home printed Performance's ending value ($355,152, Vanguard's $838 uninvested cash included) under 'YOUR INVESTMENTS'; his definition DEC-0457 says investments do not include cash, and MK-XS-M-003 is one figure on Home and Net worth ($354,314). My batch 2 choice reversed; its decision row marked replaced.</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>DONE — outside_networth_02.test.tsx renders both values; fcc_agreement pins each figure to its door.</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>src/screens/HomeScreen.tsx · src/screens/__tests__/outside_networth_02.test.tsx · src/screens/__tests__/fcc_agreement.test.tsx</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>Home is outside build 55's scope; fixed because the figure was wrong against his definition.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F225"/>
+  <autoFilter ref="A1:F226"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
One last outside test of the whole Net worth module, written for OpenAI
His words, 2026-10-09: "write one last brief for Open AI to run one last set of test across entire NW
module to ensure all fixes are in, and all screens, and functions meet tenants." build-outside-test-cards.py
gains --module-audit: from the code as it stands, the tenets; four jobs (formula check and five cases for
every function; each decided rule HELD or NOT HELD; each screen figure against the tenets); his settled
rulings (A47 replaced by DEC-3390; his class-list and investments rulings added); the 67 rules decided in
the outside reviews and in force, from the decision log; the 71 figures the Net worth screens print, from
the figure register; 101 function cards in four parts. DEC-2484b's wording refined to DEC-3390. Tracker
row. 4,105 tests green; gates exit 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$228</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$229</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F228"/>
+  <dimension ref="A1:F229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7323,8 +7323,40 @@
         </is>
       </c>
     </row>
+    <row r="229" ht="60" customHeight="1">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>Final outside test of the whole Net worth module — brief for OpenAI</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>His words, 2026-10-09: 'write one last brief for Open AI to run one last set of test across entire NW module to ensure all fixes are in, and all screens, and functions meet tenants.' Written from the code as it stands (build-outside-test-cards.py --module-audit NW --for OpenAI): the tenets; four jobs (formula check and five cases for every function; each decided rule HELD or NOT; each screen figure against the tenets); his settled rulings (A47 replaced by DEC-3390); the 67 rules decided in the outside reviews, in force, from the decision log; the 71 figures the Net worth screens print, from the figure register; 101 function cards in four parts.</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>WAITING ON HIM — to send to OpenAI</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/audit/outside-test-cases/to-send/moneykeel_audit_module_nw_for-openai_v01.md + _cards-part-1..4-of-4.md</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>Batch 06's full 60-case JSON was never returned — only its fix brief; the brief's 23 tests are in. Tenets are draft v01, not yet approved by him.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F228"/>
+  <autoFilter ref="A1:F229"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Files brought level with the decisions of 2026-10-10/11: classed-and-counted standard §14 (DEC-4036, 4059, 4082, 4105, 4327, 4350, 4528, 4529), the drawing-correction rule in the screen standard, canon term 21 'Add your debts ›', design record (account page needs a redraw), tracker rows (final audit done, re-run brief ready, drawing check, account-page redraw, Performance paused, inputs-and-use audit)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$232</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$236</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F232"/>
+  <dimension ref="A1:F236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7451,8 +7451,132 @@
         </is>
       </c>
     </row>
+    <row r="233" ht="60" customHeight="1">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>Net worth line-by-line drawing check v02 (against c40588f3, then 1769410f)</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>Every Net worth screen and state against its approved drawing and READ THIS FIRST rows; fix what the code gets wrong; correct the drawings' own errors by dated lines (DEC-4529).</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-11 — 10 code fixes over two runs; 8 correction lines on 4 drawings; empty Debts door 'Add your debts ›' (DEC-4528); a home's edit sheet no longer asks what it is invested in</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/audit/moneykeel_audit_mock-match_networth_2026-10-11_v02.md</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>The account page (Performance v17 frame 2) does NOT match: nine elements differ and the drawing's own figures do not add up ($52,704 of categories vs $101,000). Needs a redraw before it is rebuilt — next Net worth task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="45" customHeight="1">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>Account page: redraw Performance v17 frame 2 so its figures add up, then rebuild the page to it</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>Draw from the code's census strings and tokens; one phone, final state; his approval; then rebuild and mock-match.</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — next Net worth task</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/networth-and-performance/moneykeel_pres_mock_performance_v17.html</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr"/>
+    </row>
+    <row r="235" ht="60" customHeight="1">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>Claude's outside audit of Performance (4 batches, 225 cases, 45 functions incl. the time-weighted-return engine)</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>Run every case against the app; fix what his existing rules settle; bring the rest to him one at a time — AFTER Net worth is launch-ready (his order, 2026-10-11).</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>PAUSED by his order (one module at a time) — 225 of 225 run: 170 pass; 40 app errors fixed under his rules; open: 6 decision points (unknown window name, prices starting late, the trend function, partly matched sale, typed balance missing on the last record day; 0% CD settled by his rule), whether a holding's return includes its dividends, and the Home market line's 'including dividends' wording</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/audit/outside-test-cases/returned/results/performance_claude_0{1..4}_results.json</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>Briefs v02 in to-send/moneykeel_brief_performance_0N_claude-code_v02.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="60" customHeight="1">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>Read-only audit of every function's inputs and use (his objectives a and b)</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>Every input entered, decided, published, fed or derived; every function, orchestrator and metric used on a live screen.</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-11 — findings to act on module by module (Net worth first)</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/audit/moneykeel_audit_inputs-and-use_v01.xlsx · …_summary_v01.md</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>Net worth: option contract size (MK-XS-I-063) set by nothing; 6% / 7% / ±1% with no decision (MK-NW-F-034, F-040, F-064); 10 tests-only and 2 unused functions; 7 figures printed under another ID.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F232"/>
+  <autoFilter ref="A1:F236"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Performance: build the 2026-10-12 decisions DEC-4640..4646
1 unknown window name gives no figure (DEC-4640); 'Since' now starts on the record's first day, not today
2 'Prices for this holding go back…' sentence wherever a holding's window figure shows (DEC-4641)
3 retire MK-PF-F-003/016/017/018/019/021, replaced by MK-NW-O-006/008 and the daily-value graph (DEC-4642)
4 a sale bigger than recorded purchases counts once, unknown part named (DEC-4643)
5 outside case on a typed balance marked judge error, +2.00% pinned
6 a holding's return counts dividends once (DEC-4644)
7 market figure includes dividends and interest: false 'price only' records corrected, his Home wording kept (DEC-4645)
8 option contract size: broker mini flag = 10, hand-typed 'Shares per contract' default 100 (DEC-4646)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$236</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$237</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F236"/>
+  <dimension ref="A1:F237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7524,7 +7524,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>PAUSED by his order (one module at a time) — 225 of 225 run: 170 pass; 40 app errors fixed under his rules; open: 6 decision points (unknown window name, prices starting late, the trend function, partly matched sale, typed balance missing on the last record day; 0% CD settled by his rule), whether a holding's return includes its dividends, and the Home market line's 'including dividends' wording</t>
+          <t>IN PROGRESS — his answers of 2026-10-12 built (DEC-4640 … DEC-4646): the 6 decision points and the two dividend questions are closed — unknown window name refuses, prices starting late are measured and named, six unused functions removed, a partly matched sale counted once, the typed-balance case was the judge's double count (withdrawn), a holding's return carries its dividends once, the market figure's record corrected, option shares per contract</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>Briefs v02 in to-send/moneykeel_brief_performance_0N_claude-code_v02.md.</t>
+          <t>Briefs v02 in to-send/moneykeel_brief_performance_0N_claude-code_v02.md. 2026-10-12: 35 outside cases settled or removed (1 + 3 + 25 removed + 5 re-pointed + 1 + 1 + 1 brief wrong); results files carry a 'settled' line on each. Not committed.</t>
         </is>
       </c>
     </row>
@@ -7571,12 +7571,44 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>Net worth: option contract size (MK-XS-I-063) set by nothing; 6% / 7% / ±1% with no decision (MK-NW-F-034, F-040, F-064); 10 tests-only and 2 unused functions; 7 figures printed under another ID.</t>
+          <t>Net worth: option contract size (MK-XS-I-063) set by nothing; 6% / 7% / ±1% with no decision (MK-NW-F-034, F-040, F-064); 10 tests-only and 2 unused functions; 7 figures printed under another ID. 2026-10-12: option contract size (MK-XS-I-063) now set by the broker (mini option 10) or the person (DEC-4646); MK-PF-F-003 / 016 / 017 / 018 / 019 / 021 removed (DEC-4642).</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="60" customHeight="1">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>Performance decisions of 2026-10-12 — eight items, built (his: "1, 2 - approved." · "3,4, 8-approved.")</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>1 unknown window name refuses (DEC-4640) · 2 prices starting late: measured from the first price, the line wherever the figure shows (DEC-4641) · 3 six unused functions removed (DEC-4642) · 4 a sale bigger than the purchases counted once (DEC-4643) · 5 withdrawn: the judge double-counted the IRA (+2.00% is right) · 6 dividends counted once (DEC-4644, his existing rule) · 7 the market figure's 'price only' record corrected (DEC-4645) · 8 option shares per contract (DEC-4646)</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-12 — code, tests, function rules, standards, changelog, drawings' READ THIS FIRST lines; not committed</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>src/screens/__tests__/performance_decisions_2026_10_12.test.tsx · src/domain/performance/start_date_month_end.test.ts · src/domain/performance/realized.test.ts · MoneyKeel/documents/standards/moneykeel_calc_spec_precision-and-display_v01.md</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>Found while applying item 1: 'Since' was read as today, so each holding's Since figure (the category returns under the walk) was one day's move. Since now hands over its own first day.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F236"/>
+  <autoFilter ref="A1:F237"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Performance: line-by-line drawing check against v17 phones 1,3,4,5, Look back and Holding detail — 13 code fixes, account-bar arrows on one right edge, 2 READ THIS FIRST rows
Audit: MoneyKeel/documents/audit/moneykeel_audit_mock-match_performance_2026-10-12_v01.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$237</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$238</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F237"/>
+  <dimension ref="A1:F238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7607,8 +7607,40 @@
         </is>
       </c>
     </row>
+    <row r="238" ht="60" customHeight="1">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>Performance line-by-line drawing check (v17 phones 1, 3, 4, 5 · Look back v01 · Holding detail v02), against 02adb375</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>Every visible word AND figure of each phone against the screen rendered on the drawing's own day; then colours, sizes, weights; fix what the code gets wrong, each with a test; drawing arithmetic checked (DEC-4529). Phone 2, the account page, is out of scope: it is the redraw row of 2026-10-11.</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-12 — 11 code fixes (window control colours, one-line notes, 13-point date and labels, walk weights, withdrawals not red, notes' grey, category table, graph dates over a year, gridlines that hold the line, day-one frame, Holding liquidated colour); no drawing arithmetic error found; not committed</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/audit/moneykeel_audit_mock-match_performance_2026-10-12_v01.md · src/screens/__tests__/perf_mock_match_2026_10_12.test.tsx</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>Phones 1 and 3 now match the drawing figure for figure, not only word for word: the test builds a household whose record gives the drawn $100,000 → $123,000, +0.41%, +4.90%, 7.46%, 6.88%, $38,000 → $52,704 and the rest.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F237"/>
+  <autoFilter ref="A1:F238"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
DEC-5068 (Wealth generated and Return from holdings with a price history; the rest named) and DEC-5136 (walk title is always HOW $X BECAME $Y); DEC-3656 part 2 retired
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$238</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$240</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F238"/>
+  <dimension ref="A1:F240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7639,8 +7639,72 @@
         </is>
       </c>
     </row>
+    <row r="239" ht="60" customHeight="1">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>DEC-5068 — Wealth generated and Return for every holding with a history, where the beginning is worked back (his ruling of 2026-10-13)</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>thePerformance keeps the walk and leaves out a holding with no price history; Return = the holdings with a history only; notIncludedSentence replaces cannotWorkBackSentence; account page and Performance cards print it; outside cases settled; rules, standard, Changelog, v17 note.</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-13 — built and tested; Return shown where the beginning is worked back; sentence on the account page and each account's card; not committed</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/functions/networth-and-performance/dec_worked_back_known_holdings.test.ts · src/screens/__tests__/dec_worked_back_known_holdings.test.tsx · MoneyKeel/documents/networth-and-performance/moneykeel_pres_mock_performance_v17.html</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>$50,000 = VTI $40,000 (+10%) + Treasury 2031 $10,000 → Wealth generated $3,636, Return +10.00%, walk drawn (was —, —, no walk). Replaces DEC-3656 part 2 (DEC-3656b, now not in use).</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="60" customHeight="1">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>DEC-5136 — the walk card's title is always HOW $&lt;beginning&gt; BECAME $&lt;ending&gt; · ALL ACCOUNTS (his ruling of 2026-10-13)</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>Both screens title the walk the one way in every state; retire the day-one title from code, tests and mock-match expectations; READ THIS FIRST rows; Changelog.</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-13 — built and tested on both screens; READ THIS FIRST rows on v17 and Ways to add v10; not committed</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>src/screens/PerformanceScreen.tsx · src/screens/AccountPortfolioScreen.tsx · src/screens/__tests__/perf_matches_v17.test.tsx · src/screens/__tests__/perf_mock_match_2026_10_12.test.tsx</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>Day one reads HOW $354,314 BECAME $354,314 · ALL ACCOUNTS (was HOW TODAY'S VALUE STANDS · ALL ACCOUNTS $354,314); the account page gains · THIS ACCOUNT as v17 frame 2 draws it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F238"/>
+  <autoFilter ref="A1:F240"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
DEC-5291: a window that starts before the daily record is worked back from each holding's price history (replaces DEC-3035i greying); the left-out holdings named; refusal kept only where no holding has a history
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$240</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$241</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F240"/>
+  <dimension ref="A1:F241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7703,8 +7703,40 @@
         </is>
       </c>
     </row>
+    <row r="241" ht="60" customHeight="1">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>DEC-5291 — let price history count: a window that starts before the daily record is worked back, not greyed (his "approved." of 2026-10-13)</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>thePerformance works back a record-too-late window when a holding has a history (DEC-3035i's refusal only where none has); mixed accounts = the cards added up; cash gains $0 unnamed; day-one line; tests settled; rules re-read, standards, Changelog, v17 READ THIS FIRST row.</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-13 — built and tested; Performance tab, account page and Home work a too-late window back from price history; DEC-3035i marked OLD, NOT IN USE; not committed</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/functions/networth-and-performance/dec_price_history_counts.test.ts · src/screens/__tests__/dec_price_history_counts.test.tsx · MoneyKeel/documents/networth-and-performance/moneykeel_pres_mock_performance_v17.html</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>Vanguard linked today, VTI $40,000 (+10%) + Treasury 2031 $10,000 by hand: 1Y +10.00% (was greyed —), Wealth generated $3,636, Return +10.00%, sentence names Treasury 2031 (was "The record begins Oct 13, 2026, …"). Mixed: Fidelity $100,000→$112,000 + Vanguard worked back → summary $136,364→$152,000, +11.47% = the cards added up. Day-one line: "Day one: your value is real and your daily record starts today. Longer windows are worked back from each holding's price history."</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F240"/>
+  <autoFilter ref="A1:F241"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Net worth: approved day-one wording ("You added your accounts today…"); inputs-and-use audit fixes — unused monthly-history input and MK-NW-M-003 retired, old rentalIncome moved once into the rent list (MK-CF-F-216..218), figures printed under their own IDs, four never-called saved-account functions retired; account-page drawing v01 for approval
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$241</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$242</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F241"/>
+  <dimension ref="A1:F242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7731,12 +7731,44 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>Vanguard linked today, VTI $40,000 (+10%) + Treasury 2031 $10,000 by hand: 1Y +10.00% (was greyed —), Wealth generated $3,636, Return +10.00%, sentence names Treasury 2031 (was "The record begins Oct 13, 2026, …"). Mixed: Fidelity $100,000→$112,000 + Vanguard worked back → summary $136,364→$152,000, +11.47% = the cards added up. Day-one line: "Day one: your value is real and your daily record starts today. Longer windows are worked back from each holding's price history."</t>
+          <t>Vanguard linked today, VTI $40,000 (+10%) + Treasury 2031 $10,000 by hand: 1Y +10.00% (was greyed —), Wealth generated $3,636, Return +10.00%, sentence names Treasury 2031 (was "The record begins Oct 13, 2026, …"). Mixed: Fidelity $100,000→$112,000 + Vanguard worked back → summary $136,364→$152,000, +11.47% = the cards added up. Day-one line, in his words (DEC-5425, 2026-10-14): "You added your accounts today. Figures for 1M, 1Y and longer come from each holding's past prices." (the wording first proposed here was replaced)</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="60" customHeight="1">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>DEC-5425 — the Performance tab's day-one line in his words (his "approved." of 2026-10-14)</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>PerformanceScreen day-one line (where a window is worked back) reads his words; tests moved; DEC-5291's records re-quoted; standards; Changelog row; v17 READ THIS FIRST row.</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-14 — built and tested; not committed</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>src/screens/PerformanceScreen.tsx · src/screens/__tests__/dec_price_history_counts.test.tsx · src/screens/__tests__/perf_matches_v17.test.tsx · src/screens/__tests__/perf_mock_match_2026_10_12.test.tsx · MoneyKeel/documents/networth-and-performance/moneykeel_pres_mock_performance_v17.html</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>Before: "Day one: your value is real and your daily record starts today. Longer windows are worked back from each holding's price history." Now: "You added your accounts today. Figures for 1M, 1Y and longer come from each holding's past prices." Canon checked: no clash.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F241"/>
+  <autoFilter ref="A1:F242"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
DEC-5758: 8 test-only Net worth functions removed and retired (MK-NW-F-006/013/015/017/018/019/020/038); no-accounts Net worth matches v08 state C, retirement line names the missing answers (DEC-0086); account-page drawing state E (bond with the rates card)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -3445,14 +3445,14 @@
           <t>Claude: draw it in the Net worth series (v09) for approval before building.</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
-        <is>
-          <t>TO DO</t>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-18 — built and tested (commit 42048261 for the one door; the rest of state C not committed)</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>src/screens/NetWorthScreen.tsx (seeded, no accounts) · src/screens/__tests__/empty_state_q48.test.tsx</t>
+          <t>src/screens/NetWorthScreen.tsx · src/screens/__tests__/nw_no_accounts_one_door.test.tsx · src/screens/__tests__/empty_state_q48.test.tsx</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -3460,7 +3460,11 @@
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Before: a later visit with no account showed "Add your accounts ›" 3 times (hero, Cash, Investments), no Personal property, no emergency fund line, a dated title, and "＋ Add an account". Now: the same screen as the first day, Net worth v08 state C, word for word — "Add your accounts ›" once, the three ways to add once, "Add your debts" on Debts (DEC-4528). Ruled by DEC-0227. No new drawing: v08 state C is the approved drawing of this data state. The retirement line keeps state C's words only when all three answers are missing; with one or two given it names what is left (DEC-0086), e.g. "a sample, not your number — 2 answers make it yours: what you spend and what you have ›".</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="60" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
@@ -7571,7 +7575,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>Net worth: option contract size (MK-XS-I-063) set by nothing; 6% / 7% / ±1% with no decision (MK-NW-F-034, F-040, F-064); 10 tests-only and 2 unused functions; 7 figures printed under another ID. 2026-10-12: option contract size (MK-XS-I-063) now set by the broker (mini option 10) or the person (DEC-4646); MK-PF-F-003 / 016 / 017 / 018 / 019 / 021 removed (DEC-4642).</t>
+          <t>Net worth: option contract size (MK-XS-I-063) set by nothing; 6% / 7% / ±1% with no decision (MK-NW-F-034, F-040, F-064); 10 tests-only and 2 unused functions; 7 figures printed under another ID. 2026-10-12: option contract size (MK-XS-I-063) now set by the broker (mini option 10) or the person (DEC-4646); MK-PF-F-003 / 016 / 017 / 018 / 019 / 021 removed (DEC-4642). 2026-10-19: MK-NW-F-006 / 013 / 015 / 017 / 018 / 019 / 020 / 038 removed and their numbers retired (DEC-5758, his words: "Removing #4,5,6,7-10,11 - approved.") — 8 of 8.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DEC-6412: a window starting before the daily record chains price history (the gap) with the measured record — state A 1Y = Since +8.26%; one date writer for every stored date on Net worth screens (guard test)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_plan_workplan_v01.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Workplan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Workplan'!$A$1:$F$243</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F242"/>
+  <dimension ref="A1:F243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7771,8 +7771,40 @@
         </is>
       </c>
     </row>
+    <row r="243" ht="60" customHeight="1">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>DEC-6412 — a window that opens before the daily record begins is joined at the record's first day (his "approved." of 2026-10-19, amends DEC-5291)</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>thePerformance joins the days before the record (price history) to the record's own return; every caller hands over the price histories; the note under the summary; tests for the three cases and a mixed one; account-page drawing state A, side column, READ THIS FIRST row 43; Performance v17 READ THIS FIRST row; standards; Changelog row; function rules re-read.</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-19 — built and tested; not committed</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>MoneyKeel/functions/networth-and-performance/performance.ts · MoneyKeel/functions/networth-and-performance/dec6412_join_at_record_start.test.ts · src/screens/AccountPortfolioScreen.tsx · src/screens/PerformanceScreen.tsx · src/screens/HomeScreen.tsx · src/screens/__tests__/account_page_drawing_states.test.tsx · src/screens/__tests__/perf_mock_match_2026_10_12.test.tsx · MoneyKeel/documents/networth-and-performance/moneykeel_pres_mock_account-page_v01.html · MoneyKeel/documents/networth-and-performance/moneykeel_pres_mock_performance_v17.html</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>Before: state A 1Y +7.12%, 2Y +9.57% (worked back whole); Performance v17 phone 1 1Y +6.10%, 2Y +11.10%. Now: state A 1Y +8.26% (= Since), 2Y +10.87% a year; phone 1 1Y +7.46% (= Since), 2Y +11.81% a year. States B to E unchanged.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F242"/>
+  <autoFilter ref="A1:F243"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>